<commit_message>
Schichtplaner: alle Fragen als PDF und in der Vorlage, was von LogX gebraucht wird (Runde 206)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DT8NfaHWD2WwmwkipPurng
</commit_message>
<xml_diff>
--- a/vorlagen/Schichtplaner-Vorlage.xlsx
+++ b/vorlagen/Schichtplaner-Vorlage.xlsx
@@ -61,13 +61,13 @@
     </font>
     <font>
       <name val="Calibri"/>
-      <b val="1"/>
+      <i val="1"/>
+      <color rgb="0064748B"/>
       <sz val="11"/>
     </font>
     <font>
       <name val="Calibri"/>
-      <i val="1"/>
-      <color rgb="0064748B"/>
+      <b val="1"/>
       <sz val="11"/>
     </font>
   </fonts>
@@ -120,7 +120,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -136,14 +136,17 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -670,13 +673,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D21"/>
+  <dimension ref="A1:E25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
-    <col width="24" customWidth="1" min="2" max="2"/>
-    <col width="70" customWidth="1" min="3" max="3"/>
-    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="62" customWidth="1" min="3" max="3"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
+    <col width="50" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1">
@@ -697,6 +701,11 @@
       </c>
       <c r="D1" s="4" t="inlineStr">
         <is>
+          <t>Heute in der App</t>
+        </is>
+      </c>
+      <c r="E1" s="4" t="inlineStr">
+        <is>
           <t>Antwort</t>
         </is>
       </c>
@@ -707,15 +716,20 @@
       </c>
       <c r="B2" s="6" t="inlineStr">
         <is>
-          <t>Studios und Öffnungszeiten</t>
+          <t>A · Ohne diese Angaben gibt es keinen Plan</t>
         </is>
       </c>
       <c r="C2" s="6" t="inlineStr">
         <is>
-          <t>Welche Öffnungszeiten hat jedes der 14 Studios an welchem Wochentag? (Die Namen stehen schon im Excel – bitte prüfen.) Bitte im Excel im Blatt „Studios“ eintragen.</t>
-        </is>
-      </c>
-      <c r="D2" s="7" t="n"/>
+          <t>Welche Studios sollen im ersten Monat mitgeplant werden – alle 14 oder zum Testen erst eins oder zwei?</t>
+        </is>
+      </c>
+      <c r="D2" s="7" t="inlineStr">
+        <is>
+          <t>Empfehlung: erst ein Studio.</t>
+        </is>
+      </c>
+      <c r="E2" s="8" t="n"/>
     </row>
     <row r="3" ht="48" customHeight="1">
       <c r="A3" s="5" t="n">
@@ -723,15 +737,20 @@
       </c>
       <c r="B3" s="6" t="inlineStr">
         <is>
-          <t>Studios und Öffnungszeiten</t>
+          <t>A · Ohne diese Angaben gibt es keinen Plan</t>
         </is>
       </c>
       <c r="C3" s="6" t="inlineStr">
         <is>
-          <t>An welchen Feiertagen sind die Studios zu? Gibt es Betriebsferien?</t>
-        </is>
-      </c>
-      <c r="D3" s="7" t="n"/>
+          <t>Öffnungszeiten je Studio und Wochentag.</t>
+        </is>
+      </c>
+      <c r="D3" s="7" t="inlineStr">
+        <is>
+          <t>Ins Excel, Blatt „Studios“.</t>
+        </is>
+      </c>
+      <c r="E3" s="8" t="n"/>
     </row>
     <row r="4" ht="48" customHeight="1">
       <c r="A4" s="5" t="n">
@@ -739,15 +758,20 @@
       </c>
       <c r="B4" s="6" t="inlineStr">
         <is>
-          <t>Schichten und Besetzung</t>
+          <t>A · Ohne diese Angaben gibt es keinen Plan</t>
         </is>
       </c>
       <c r="C4" s="6" t="inlineStr">
         <is>
-          <t>Gibt es feste Schichten (z. B. Früh 7–14 Uhr, Spät 14–21 Uhr) oder wechselnde Zeiten? Sind sie in allen Studios gleich? Bitte im Excel im Blatt „Schichten“ eintragen.</t>
-        </is>
-      </c>
-      <c r="D4" s="7" t="n"/>
+          <t>Schichten je Studio: Name, Beginn, Ende, an welchen Wochentagen. Sind sie in allen Studios gleich?</t>
+        </is>
+      </c>
+      <c r="D4" s="7" t="inlineStr">
+        <is>
+          <t>Ins Excel, Blatt „Schichten“. Heute in der Demo: Früh 7–14, Spät 14–21, Samstag 9–14.</t>
+        </is>
+      </c>
+      <c r="E4" s="8" t="n"/>
     </row>
     <row r="5" ht="48" customHeight="1">
       <c r="A5" s="5" t="n">
@@ -755,15 +779,20 @@
       </c>
       <c r="B5" s="6" t="inlineStr">
         <is>
-          <t>Schichten und Besetzung</t>
+          <t>A · Ohne diese Angaben gibt es keinen Plan</t>
         </is>
       </c>
       <c r="C5" s="6" t="inlineStr">
         <is>
-          <t>Wie viele Leute müssen mindestens gleichzeitig im Studio sein? Gibt es Zeiten, Tage oder Studios, an denen es mehr sein müssen (Stoßzeiten)?</t>
-        </is>
-      </c>
-      <c r="D5" s="7" t="n"/>
+          <t>Das Team: eine Zeile pro Person – Name genau wie in der App, Hauptstudio, in welchen Studios sie aushilft, Stunden pro Woche (Minijob: Monatsgrenze).</t>
+        </is>
+      </c>
+      <c r="D5" s="7" t="inlineStr">
+        <is>
+          <t>Ins Excel, Blatt „Mitarbeiter“.</t>
+        </is>
+      </c>
+      <c r="E5" s="8" t="n"/>
     </row>
     <row r="6" ht="48" customHeight="1">
       <c r="A6" s="5" t="n">
@@ -771,15 +800,20 @@
       </c>
       <c r="B6" s="6" t="inlineStr">
         <is>
-          <t>Schichten und Besetzung</t>
+          <t>A · Ohne diese Angaben gibt es keinen Plan</t>
         </is>
       </c>
       <c r="C6" s="6" t="inlineStr">
         <is>
-          <t>Wer darf nicht allein im Studio sein – nur Azubis und Neue, oder auch bestimmte Personen? Und wer zählt als „Begleitung“, damit diese Person nicht mehr allein ist?</t>
-        </is>
-      </c>
-      <c r="D6" s="7" t="n"/>
+          <t>Wer kann wann grundsätzlich nicht? (z. B. „nie Dienstag“, „nur früh“, „Di Uni“)</t>
+        </is>
+      </c>
+      <c r="D6" s="7" t="inlineStr">
+        <is>
+          <t>Ins Excel, Blatt „Mitarbeiter“, Spalten Mo–So und „Sperrzeiten“.</t>
+        </is>
+      </c>
+      <c r="E6" s="8" t="n"/>
     </row>
     <row r="7" ht="48" customHeight="1">
       <c r="A7" s="5" t="n">
@@ -787,15 +821,20 @@
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>Schichten und Besetzung</t>
+          <t>B · Besetzung</t>
         </is>
       </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>Gibt es Aufgaben, die nur bestimmte Personen können (z. B. Probetraining, Kasse, Abschluss am Abend, Erste Hilfe)? Muss in jeder Schicht mindestens eine solche Person da sein?</t>
-        </is>
-      </c>
-      <c r="D7" s="7" t="n"/>
+          <t>Wie viele Personen müssen mindestens gleichzeitig im Studio sein?</t>
+        </is>
+      </c>
+      <c r="D7" s="7" t="inlineStr">
+        <is>
+          <t>Heute: 1 je Schicht.</t>
+        </is>
+      </c>
+      <c r="E7" s="8" t="n"/>
     </row>
     <row r="8" ht="48" customHeight="1">
       <c r="A8" s="5" t="n">
@@ -803,15 +842,20 @@
       </c>
       <c r="B8" s="6" t="inlineStr">
         <is>
-          <t>Schichten und Besetzung</t>
+          <t>B · Besetzung</t>
         </is>
       </c>
       <c r="C8" s="6" t="inlineStr">
         <is>
-          <t>Werden Regionalleiter mit in den Plan eingeteilt, oder stehen sie nur bei Bedarf zur Verfügung?</t>
-        </is>
-      </c>
-      <c r="D8" s="7" t="n"/>
+          <t>Gibt es Stoßzeiten, Tage oder Studios, an denen mehr Leute da sein müssen? Wann, wo, wie viele?</t>
+        </is>
+      </c>
+      <c r="D8" s="7" t="inlineStr">
+        <is>
+          <t>Heute: nur über „Sondertage“ für einzelne Daten.</t>
+        </is>
+      </c>
+      <c r="E8" s="8" t="n"/>
     </row>
     <row r="9" ht="48" customHeight="1">
       <c r="A9" s="5" t="n">
@@ -819,15 +863,20 @@
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>Arbeitszeit und Fairness</t>
+          <t>B · Besetzung</t>
         </is>
       </c>
       <c r="C9" s="6" t="inlineStr">
         <is>
-          <t>Wie lang darf eine Schicht höchstens sein, und ab wann gibt es Pause?</t>
-        </is>
-      </c>
-      <c r="D9" s="7" t="n"/>
+          <t>Wer darf nicht allein im Studio sein (Azubis, Neue, bestimmte Personen)? Und wer zählt als Begleitung?</t>
+        </is>
+      </c>
+      <c r="D9" s="7" t="inlineStr">
+        <is>
+          <t>Heute: Begleitung ist jede Person mit „darf allein: ja“.</t>
+        </is>
+      </c>
+      <c r="E9" s="8" t="n"/>
     </row>
     <row r="10" ht="48" customHeight="1">
       <c r="A10" s="5" t="n">
@@ -835,15 +884,20 @@
       </c>
       <c r="B10" s="6" t="inlineStr">
         <is>
-          <t>Arbeitszeit und Fairness</t>
+          <t>B · Besetzung</t>
         </is>
       </c>
       <c r="C10" s="6" t="inlineStr">
         <is>
-          <t>Wie viele Tage am Stück darf jemand höchstens arbeiten? Gibt es feste freie Tage?</t>
-        </is>
-      </c>
-      <c r="D10" s="7" t="n"/>
+          <t>Muss in bestimmten Schichten jemand mit einer bestimmten Fähigkeit da sein (Probetraining, Kasse, Abschluss am Abend, Erste Hilfe)? In welchen?</t>
+        </is>
+      </c>
+      <c r="D10" s="7" t="inlineStr">
+        <is>
+          <t>Heute: je Schicht eine Fähigkeit („Braucht jemanden mit …“).</t>
+        </is>
+      </c>
+      <c r="E10" s="8" t="n"/>
     </row>
     <row r="11" ht="48" customHeight="1">
       <c r="A11" s="5" t="n">
@@ -851,15 +905,20 @@
       </c>
       <c r="B11" s="6" t="inlineStr">
         <is>
-          <t>Arbeitszeit und Fairness</t>
+          <t>B · Besetzung</t>
         </is>
       </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
-          <t>Wie werden Wochenenden und Feiertage verteilt – reihum, oder hat jemand fest frei?</t>
-        </is>
-      </c>
-      <c r="D11" s="7" t="n"/>
+          <t>Werden Studioleitungen und Regionalleiter fest eingeplant oder nur bei Bedarf?</t>
+        </is>
+      </c>
+      <c r="D11" s="7" t="inlineStr">
+        <is>
+          <t>Heute: wie alle anderen, wenn sie im Blatt „Mitarbeiter“ stehen.</t>
+        </is>
+      </c>
+      <c r="E11" s="8" t="n"/>
     </row>
     <row r="12" ht="48" customHeight="1">
       <c r="A12" s="5" t="n">
@@ -867,15 +926,20 @@
       </c>
       <c r="B12" s="6" t="inlineStr">
         <is>
-          <t>Arbeitszeit und Fairness</t>
+          <t>C · Arbeitszeit</t>
         </is>
       </c>
       <c r="C12" s="6" t="inlineStr">
         <is>
-          <t>Gibt es Mitarbeiter unter 18 Jahren? Für sie gelten strengere Regeln (z. B. keine späten Schichten).</t>
-        </is>
-      </c>
-      <c r="D12" s="7" t="n"/>
+          <t>Wie lang darf eine Schicht höchstens sein, und ab wann gibt es Pause?</t>
+        </is>
+      </c>
+      <c r="D12" s="7" t="inlineStr">
+        <is>
+          <t>Heute: wird nicht geprüft.</t>
+        </is>
+      </c>
+      <c r="E12" s="8" t="n"/>
     </row>
     <row r="13" ht="48" customHeight="1">
       <c r="A13" s="5" t="n">
@@ -883,15 +947,20 @@
       </c>
       <c r="B13" s="6" t="inlineStr">
         <is>
-          <t>Arbeitszeit und Fairness</t>
+          <t>C · Arbeitszeit</t>
         </is>
       </c>
       <c r="C13" s="6" t="inlineStr">
         <is>
-          <t>Minijobs: Gilt pro Person eine feste Höchstzahl an Stunden im Monat? Wenn nein: Wie hoch ist der Stundenlohn, damit die Maschine die Grenze ausrechnen kann?</t>
-        </is>
-      </c>
-      <c r="D13" s="7" t="n"/>
+          <t>Wie viele Tage am Stück darf jemand höchstens arbeiten?</t>
+        </is>
+      </c>
+      <c r="D13" s="7" t="inlineStr">
+        <is>
+          <t>Heute: 6.</t>
+        </is>
+      </c>
+      <c r="E13" s="8" t="n"/>
     </row>
     <row r="14" ht="48" customHeight="1">
       <c r="A14" s="5" t="n">
@@ -899,15 +968,20 @@
       </c>
       <c r="B14" s="6" t="inlineStr">
         <is>
-          <t>Wünsche und Konflikte</t>
+          <t>C · Arbeitszeit</t>
         </is>
       </c>
       <c r="C14" s="6" t="inlineStr">
         <is>
-          <t>Was hat Vorrang, wenn sich etwas beisst? Bitte in eine Reihenfolge bringen: Besetzung · vereinbarte Stunden · Wünsche der Mitarbeiter · Fairness.</t>
-        </is>
-      </c>
-      <c r="D14" s="7" t="n"/>
+          <t>Höchstens wie viele Tage pro Woche – für alle gleich oder je Person?</t>
+        </is>
+      </c>
+      <c r="D14" s="7" t="inlineStr">
+        <is>
+          <t>Heute: je Person im Excel, sonst ohne Grenze.</t>
+        </is>
+      </c>
+      <c r="E14" s="8" t="n"/>
     </row>
     <row r="15" ht="48" customHeight="1">
       <c r="A15" s="5" t="n">
@@ -915,15 +989,20 @@
       </c>
       <c r="B15" s="6" t="inlineStr">
         <is>
-          <t>Wünsche und Konflikte</t>
+          <t>C · Arbeitszeit</t>
         </is>
       </c>
       <c r="C15" s="6" t="inlineStr">
         <is>
-          <t>Bis wann vor dem Monat müssen die Wünsche eingetragen sein (z. B. bis zum 15. des Vormonats)?</t>
-        </is>
-      </c>
-      <c r="D15" s="7" t="n"/>
+          <t>Gibt es Mitarbeiter unter 18?</t>
+        </is>
+      </c>
+      <c r="D15" s="7" t="inlineStr">
+        <is>
+          <t>Wenn ja, gilt automatisch: nur 6–20 Uhr, höchstens 8 Stunden.</t>
+        </is>
+      </c>
+      <c r="E15" s="8" t="n"/>
     </row>
     <row r="16" ht="48" customHeight="1">
       <c r="A16" s="5" t="n">
@@ -931,15 +1010,20 @@
       </c>
       <c r="B16" s="6" t="inlineStr">
         <is>
-          <t>Wünsche und Konflikte</t>
+          <t>C · Arbeitszeit</t>
         </is>
       </c>
       <c r="C16" s="6" t="inlineStr">
         <is>
-          <t>Wie viele Wunsch-frei-Tage darf jeder pro Monat angeben?</t>
-        </is>
-      </c>
-      <c r="D16" s="7" t="n"/>
+          <t>Feiertage in NRW: geschlossen oder offen? Gibt es Betriebsferien?</t>
+        </is>
+      </c>
+      <c r="D16" s="7" t="inlineStr">
+        <is>
+          <t>Heute: offen (umschaltbar).</t>
+        </is>
+      </c>
+      <c r="E16" s="8" t="n"/>
     </row>
     <row r="17" ht="48" customHeight="1">
       <c r="A17" s="5" t="n">
@@ -947,15 +1031,20 @@
       </c>
       <c r="B17" s="6" t="inlineStr">
         <is>
-          <t>Wünsche und Konflikte</t>
+          <t>D · Wünsche und Fairness</t>
         </is>
       </c>
       <c r="C17" s="6" t="inlineStr">
         <is>
-          <t>Wenn eine Schicht nicht zu besetzen ist: Soll die Maschine nur die Lücke melden oder gleich vorschlagen, wen man fragen könnte?</t>
-        </is>
-      </c>
-      <c r="D17" s="7" t="n"/>
+          <t>Bis zum wievielten des Vormonats müssen Wünsche eingetragen sein?</t>
+        </is>
+      </c>
+      <c r="D17" s="7" t="inlineStr">
+        <is>
+          <t>Heute: bis zum 15.</t>
+        </is>
+      </c>
+      <c r="E17" s="8" t="n"/>
     </row>
     <row r="18" ht="48" customHeight="1">
       <c r="A18" s="5" t="n">
@@ -963,15 +1052,20 @@
       </c>
       <c r="B18" s="6" t="inlineStr">
         <is>
-          <t>Ablauf und LogX</t>
+          <t>D · Wünsche und Fairness</t>
         </is>
       </c>
       <c r="C18" s="6" t="inlineStr">
         <is>
-          <t>Wer prüft und veröffentlicht den Plan – nur Sie, oder auch die Studioleiter für ihre Studios?</t>
-        </is>
-      </c>
-      <c r="D18" s="7" t="n"/>
+          <t>Wie viele Wunsch-frei-Tage darf jede Person im Monat angeben?</t>
+        </is>
+      </c>
+      <c r="D18" s="7" t="inlineStr">
+        <is>
+          <t>Heute: keine Grenze.</t>
+        </is>
+      </c>
+      <c r="E18" s="8" t="n"/>
     </row>
     <row r="19" ht="48" customHeight="1">
       <c r="A19" s="5" t="n">
@@ -979,15 +1073,20 @@
       </c>
       <c r="B19" s="6" t="inlineStr">
         <is>
-          <t>Ablauf und LogX</t>
+          <t>D · Wünsche und Fairness</t>
         </is>
       </c>
       <c r="C19" s="6" t="inlineStr">
         <is>
-          <t>Wie weit im Voraus soll der Plan fertig sein (z. B. am 20. für den nächsten Monat)?</t>
-        </is>
-      </c>
-      <c r="D19" s="7" t="n"/>
+          <t>Was hat Vorrang, wenn es sich beisst? Bitte in eine Reihenfolge: Besetzung · vereinbarte Stunden · Wünsche · Fairness.</t>
+        </is>
+      </c>
+      <c r="D19" s="7" t="inlineStr">
+        <is>
+          <t>Heute: Besetzung zuerst; ein Wunsch wird nur als Rückfrage gebrochen.</t>
+        </is>
+      </c>
+      <c r="E19" s="8" t="n"/>
     </row>
     <row r="20" ht="48" customHeight="1">
       <c r="A20" s="5" t="n">
@@ -995,15 +1094,20 @@
       </c>
       <c r="B20" s="6" t="inlineStr">
         <is>
-          <t>Ablauf und LogX</t>
+          <t>D · Wünsche und Fairness</t>
         </is>
       </c>
       <c r="C20" s="6" t="inlineStr">
         <is>
-          <t>Wie wird heute in LogX eingetragen? Hilfreich wären Bildschirmfotos und ein exportierter alter Plan.</t>
-        </is>
-      </c>
-      <c r="D20" s="7" t="n"/>
+          <t>Wochenenden: reihum verteilen, oder hat jemand fest frei?</t>
+        </is>
+      </c>
+      <c r="D20" s="7" t="inlineStr">
+        <is>
+          <t>Heute: reihum, so gleich wie möglich.</t>
+        </is>
+      </c>
+      <c r="E20" s="8" t="n"/>
     </row>
     <row r="21" ht="48" customHeight="1">
       <c r="A21" s="5" t="n">
@@ -1011,15 +1115,104 @@
       </c>
       <c r="B21" s="6" t="inlineStr">
         <is>
-          <t>Ablauf und LogX</t>
+          <t>D · Wünsche und Fairness</t>
         </is>
       </c>
       <c r="C21" s="6" t="inlineStr">
         <is>
-          <t>Kann LogX Dateien importieren oder exportieren (Excel/CSV)? Gibt es eine Mitarbeiterliste zum Exportieren?</t>
-        </is>
-      </c>
-      <c r="D21" s="7" t="n"/>
+          <t>Fällt jemand aus: nur die Lücke melden oder gleich vorschlagen, wen man fragen kann?</t>
+        </is>
+      </c>
+      <c r="D21" s="7" t="inlineStr">
+        <is>
+          <t>Heute: bis zu drei Vorschläge.</t>
+        </is>
+      </c>
+      <c r="E21" s="8" t="n"/>
+    </row>
+    <row r="22" ht="48" customHeight="1">
+      <c r="A22" s="5" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" s="6" t="inlineStr">
+        <is>
+          <t>E · Ablauf</t>
+        </is>
+      </c>
+      <c r="C22" s="6" t="inlineStr">
+        <is>
+          <t>Wer erstellt und veröffentlicht den Plan – nur die Geschäftsführung oder auch die Studioleitung für ihr Studio?</t>
+        </is>
+      </c>
+      <c r="D22" s="7" t="inlineStr">
+        <is>
+          <t>Heute: nur die Geschäftsführung.</t>
+        </is>
+      </c>
+      <c r="E22" s="8" t="n"/>
+    </row>
+    <row r="23" ht="48" customHeight="1">
+      <c r="A23" s="5" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" s="6" t="inlineStr">
+        <is>
+          <t>E · Ablauf</t>
+        </is>
+      </c>
+      <c r="C23" s="6" t="inlineStr">
+        <is>
+          <t>Bis wann muss der Plan für den nächsten Monat fertig sein (z. B. am 20.)?</t>
+        </is>
+      </c>
+      <c r="D23" s="7" t="inlineStr">
+        <is>
+          <t>Heute: keine Frist.</t>
+        </is>
+      </c>
+      <c r="E23" s="8" t="n"/>
+    </row>
+    <row r="24" ht="48" customHeight="1">
+      <c r="A24" s="5" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" s="6" t="inlineStr">
+        <is>
+          <t>E · Ablauf</t>
+        </is>
+      </c>
+      <c r="C24" s="6" t="inlineStr">
+        <is>
+          <t>Muss die Leitung jeden Schichttausch bestätigen?</t>
+        </is>
+      </c>
+      <c r="D24" s="7" t="inlineStr">
+        <is>
+          <t>Heute: ja.</t>
+        </is>
+      </c>
+      <c r="E24" s="8" t="n"/>
+    </row>
+    <row r="25" ht="48" customHeight="1">
+      <c r="A25" s="5" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" s="6" t="inlineStr">
+        <is>
+          <t>E · Ablauf</t>
+        </is>
+      </c>
+      <c r="C25" s="6" t="inlineStr">
+        <is>
+          <t>Wird der Plan danach noch in LogX eingetragen? (Was ich dafür brauche: letzte Seite)</t>
+        </is>
+      </c>
+      <c r="D25" s="7" t="inlineStr">
+        <is>
+          <t>Heute: „Für LogX kopieren“ legt eine Tabelle in die Zwischenablage.</t>
+        </is>
+      </c>
+      <c r="E25" s="8" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1115,7 +1308,7 @@
       </c>
     </row>
     <row r="2" ht="22" customHeight="1">
-      <c r="A2" s="8" t="inlineStr">
+      <c r="A2" s="9" t="inlineStr">
         <is>
           <t>Longerich</t>
         </is>
@@ -1132,7 +1325,7 @@
       <c r="K2" s="6" t="n"/>
     </row>
     <row r="3" ht="22" customHeight="1">
-      <c r="A3" s="8" t="inlineStr">
+      <c r="A3" s="9" t="inlineStr">
         <is>
           <t>Nippes</t>
         </is>
@@ -1149,7 +1342,7 @@
       <c r="K3" s="6" t="n"/>
     </row>
     <row r="4" ht="22" customHeight="1">
-      <c r="A4" s="8" t="inlineStr">
+      <c r="A4" s="9" t="inlineStr">
         <is>
           <t>Ebertplatz</t>
         </is>
@@ -1166,7 +1359,7 @@
       <c r="K4" s="6" t="n"/>
     </row>
     <row r="5" ht="22" customHeight="1">
-      <c r="A5" s="8" t="inlineStr">
+      <c r="A5" s="9" t="inlineStr">
         <is>
           <t>Rath</t>
         </is>
@@ -1183,7 +1376,7 @@
       <c r="K5" s="6" t="n"/>
     </row>
     <row r="6" ht="22" customHeight="1">
-      <c r="A6" s="8" t="inlineStr">
+      <c r="A6" s="9" t="inlineStr">
         <is>
           <t>Porz</t>
         </is>
@@ -1200,7 +1393,7 @@
       <c r="K6" s="6" t="n"/>
     </row>
     <row r="7" ht="22" customHeight="1">
-      <c r="A7" s="8" t="inlineStr">
+      <c r="A7" s="9" t="inlineStr">
         <is>
           <t>Rondorf</t>
         </is>
@@ -1217,7 +1410,7 @@
       <c r="K7" s="6" t="n"/>
     </row>
     <row r="8" ht="22" customHeight="1">
-      <c r="A8" s="8" t="inlineStr">
+      <c r="A8" s="9" t="inlineStr">
         <is>
           <t>Hürth</t>
         </is>
@@ -1234,7 +1427,7 @@
       <c r="K8" s="6" t="n"/>
     </row>
     <row r="9" ht="22" customHeight="1">
-      <c r="A9" s="8" t="inlineStr">
+      <c r="A9" s="9" t="inlineStr">
         <is>
           <t>Brühl</t>
         </is>
@@ -1251,7 +1444,7 @@
       <c r="K9" s="6" t="n"/>
     </row>
     <row r="10" ht="22" customHeight="1">
-      <c r="A10" s="8" t="inlineStr">
+      <c r="A10" s="9" t="inlineStr">
         <is>
           <t>Niederkassel Mondorf</t>
         </is>
@@ -1268,7 +1461,7 @@
       <c r="K10" s="6" t="n"/>
     </row>
     <row r="11" ht="22" customHeight="1">
-      <c r="A11" s="8" t="inlineStr">
+      <c r="A11" s="9" t="inlineStr">
         <is>
           <t>Refrath</t>
         </is>
@@ -1285,7 +1478,7 @@
       <c r="K11" s="6" t="n"/>
     </row>
     <row r="12" ht="22" customHeight="1">
-      <c r="A12" s="8" t="inlineStr">
+      <c r="A12" s="9" t="inlineStr">
         <is>
           <t>Overath</t>
         </is>
@@ -1302,7 +1495,7 @@
       <c r="K12" s="6" t="n"/>
     </row>
     <row r="13" ht="22" customHeight="1">
-      <c r="A13" s="8" t="inlineStr">
+      <c r="A13" s="9" t="inlineStr">
         <is>
           <t>Marialinden</t>
         </is>
@@ -1319,7 +1512,7 @@
       <c r="K13" s="6" t="n"/>
     </row>
     <row r="14" ht="22" customHeight="1">
-      <c r="A14" s="8" t="inlineStr">
+      <c r="A14" s="9" t="inlineStr">
         <is>
           <t>Rösrath</t>
         </is>
@@ -1336,7 +1529,7 @@
       <c r="K14" s="6" t="n"/>
     </row>
     <row r="15" ht="22" customHeight="1">
-      <c r="A15" s="8" t="inlineStr">
+      <c r="A15" s="9" t="inlineStr">
         <is>
           <t>Seelscheid</t>
         </is>
@@ -1353,7 +1546,7 @@
       <c r="K15" s="6" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="9" t="inlineStr">
+      <c r="A17" s="10" t="inlineStr">
         <is>
           <t>Beispiel für eine Zeile: Mo 07:00–21:00 · mindestens 1 · „Mo–Do 16–20 Uhr 2 Personen“ · „Sa nur bis 14 Uhr“</t>
         </is>
@@ -1434,112 +1627,112 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="10" t="inlineStr">
+      <c r="A2" s="11" t="inlineStr">
         <is>
           <t>alle</t>
         </is>
       </c>
-      <c r="B2" s="10" t="inlineStr">
+      <c r="B2" s="11" t="inlineStr">
         <is>
           <t>Früh</t>
         </is>
       </c>
-      <c r="C2" s="10" t="inlineStr">
+      <c r="C2" s="11" t="inlineStr">
         <is>
           <t>07:00</t>
         </is>
       </c>
-      <c r="D2" s="10" t="inlineStr">
+      <c r="D2" s="11" t="inlineStr">
         <is>
           <t>14:00</t>
         </is>
       </c>
-      <c r="E2" s="10" t="inlineStr">
+      <c r="E2" s="11" t="inlineStr">
         <is>
           <t>Mo–Fr</t>
         </is>
       </c>
-      <c r="F2" s="10" t="n">
+      <c r="F2" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="G2" s="10" t="inlineStr"/>
-      <c r="H2" s="10" t="inlineStr">
+      <c r="G2" s="11" t="inlineStr"/>
+      <c r="H2" s="11" t="inlineStr">
         <is>
           <t>Beispiel – bitte anpassen</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="10" t="inlineStr">
+      <c r="A3" s="11" t="inlineStr">
         <is>
           <t>alle</t>
         </is>
       </c>
-      <c r="B3" s="10" t="inlineStr">
+      <c r="B3" s="11" t="inlineStr">
         <is>
           <t>Spät</t>
         </is>
       </c>
-      <c r="C3" s="10" t="inlineStr">
+      <c r="C3" s="11" t="inlineStr">
         <is>
           <t>14:00</t>
         </is>
       </c>
-      <c r="D3" s="10" t="inlineStr">
+      <c r="D3" s="11" t="inlineStr">
         <is>
           <t>21:00</t>
         </is>
       </c>
-      <c r="E3" s="10" t="inlineStr">
+      <c r="E3" s="11" t="inlineStr">
         <is>
           <t>Mo–Fr</t>
         </is>
       </c>
-      <c r="F3" s="10" t="n">
+      <c r="F3" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="G3" s="10" t="inlineStr">
+      <c r="G3" s="11" t="inlineStr">
         <is>
           <t>Abschluss</t>
         </is>
       </c>
-      <c r="H3" s="10" t="inlineStr">
+      <c r="H3" s="11" t="inlineStr">
         <is>
           <t>Beispiel – bitte anpassen</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="10" t="inlineStr">
+      <c r="A4" s="11" t="inlineStr">
         <is>
           <t>alle</t>
         </is>
       </c>
-      <c r="B4" s="10" t="inlineStr">
+      <c r="B4" s="11" t="inlineStr">
         <is>
           <t>Samstag</t>
         </is>
       </c>
-      <c r="C4" s="10" t="inlineStr">
+      <c r="C4" s="11" t="inlineStr">
         <is>
           <t>09:00</t>
         </is>
       </c>
-      <c r="D4" s="10" t="inlineStr">
+      <c r="D4" s="11" t="inlineStr">
         <is>
           <t>14:00</t>
         </is>
       </c>
-      <c r="E4" s="10" t="inlineStr">
+      <c r="E4" s="11" t="inlineStr">
         <is>
           <t>Sa</t>
         </is>
       </c>
-      <c r="F4" s="10" t="n">
+      <c r="F4" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="G4" s="10" t="inlineStr"/>
-      <c r="H4" s="10" t="inlineStr">
+      <c r="G4" s="11" t="inlineStr"/>
+      <c r="H4" s="11" t="inlineStr">
         <is>
           <t>Beispiel – bitte anpassen</t>
         </is>
@@ -2079,194 +2272,194 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="10" t="inlineStr">
+      <c r="A2" s="11" t="inlineStr">
         <is>
           <t>Beispiel: Lisa M.</t>
         </is>
       </c>
-      <c r="B2" s="10" t="inlineStr">
+      <c r="B2" s="11" t="inlineStr">
         <is>
           <t>Minijob</t>
         </is>
       </c>
-      <c r="C2" s="10" t="inlineStr">
+      <c r="C2" s="11" t="inlineStr">
         <is>
           <t>Nippes</t>
         </is>
       </c>
-      <c r="D2" s="10" t="inlineStr">
+      <c r="D2" s="11" t="inlineStr">
         <is>
           <t>Longerich, Ebertplatz</t>
         </is>
       </c>
-      <c r="E2" s="10" t="inlineStr"/>
-      <c r="F2" s="10" t="n">
+      <c r="E2" s="11" t="inlineStr"/>
+      <c r="F2" s="11" t="n">
         <v>40</v>
       </c>
-      <c r="G2" s="10" t="n">
+      <c r="G2" s="11" t="n">
         <v>3</v>
       </c>
-      <c r="H2" s="10" t="inlineStr">
+      <c r="H2" s="11" t="inlineStr">
         <is>
           <t>ja</t>
         </is>
       </c>
-      <c r="I2" s="10" t="inlineStr">
+      <c r="I2" s="11" t="inlineStr">
         <is>
           <t>nein</t>
         </is>
       </c>
-      <c r="J2" s="10" t="inlineStr">
+      <c r="J2" s="11" t="inlineStr">
         <is>
           <t>Probetraining</t>
         </is>
       </c>
-      <c r="K2" s="10" t="inlineStr">
+      <c r="K2" s="11" t="inlineStr">
         <is>
           <t>nur spät</t>
         </is>
       </c>
-      <c r="L2" s="10" t="inlineStr">
+      <c r="L2" s="11" t="inlineStr">
         <is>
           <t>nie</t>
         </is>
       </c>
-      <c r="M2" s="10" t="inlineStr">
+      <c r="M2" s="11" t="inlineStr">
         <is>
           <t>nur spät</t>
         </is>
       </c>
-      <c r="N2" s="10" t="inlineStr">
+      <c r="N2" s="11" t="inlineStr">
         <is>
           <t>nie</t>
         </is>
       </c>
-      <c r="O2" s="10" t="inlineStr">
+      <c r="O2" s="11" t="inlineStr">
         <is>
           <t>ganztags</t>
         </is>
       </c>
-      <c r="P2" s="10" t="inlineStr">
+      <c r="P2" s="11" t="inlineStr">
         <is>
           <t>ganztags</t>
         </is>
       </c>
-      <c r="Q2" s="10" t="inlineStr">
+      <c r="Q2" s="11" t="inlineStr">
         <is>
           <t>nie</t>
         </is>
       </c>
-      <c r="R2" s="10" t="inlineStr"/>
-      <c r="S2" s="10" t="inlineStr">
+      <c r="R2" s="11" t="inlineStr"/>
+      <c r="S2" s="11" t="inlineStr">
         <is>
           <t>Spät</t>
         </is>
       </c>
-      <c r="T2" s="10" t="inlineStr">
+      <c r="T2" s="11" t="inlineStr">
         <is>
           <t>ja</t>
         </is>
       </c>
-      <c r="U2" s="10" t="inlineStr"/>
-      <c r="V2" s="10" t="inlineStr"/>
-      <c r="W2" s="10" t="inlineStr">
+      <c r="U2" s="11" t="inlineStr"/>
+      <c r="V2" s="11" t="inlineStr"/>
+      <c r="W2" s="11" t="inlineStr">
         <is>
           <t>samstags nur alle zwei Wochen</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="10" t="inlineStr">
+      <c r="A3" s="11" t="inlineStr">
         <is>
           <t>Beispiel: Tom K.</t>
         </is>
       </c>
-      <c r="B3" s="10" t="inlineStr">
+      <c r="B3" s="11" t="inlineStr">
         <is>
           <t>Azubi</t>
         </is>
       </c>
-      <c r="C3" s="10" t="inlineStr">
+      <c r="C3" s="11" t="inlineStr">
         <is>
           <t>Porz</t>
         </is>
       </c>
-      <c r="D3" s="10" t="inlineStr"/>
-      <c r="E3" s="10" t="n">
+      <c r="D3" s="11" t="inlineStr"/>
+      <c r="E3" s="11" t="n">
         <v>40</v>
       </c>
-      <c r="F3" s="10" t="inlineStr"/>
-      <c r="G3" s="10" t="n">
+      <c r="F3" s="11" t="inlineStr"/>
+      <c r="G3" s="11" t="n">
         <v>5</v>
       </c>
-      <c r="H3" s="10" t="inlineStr">
+      <c r="H3" s="11" t="inlineStr">
         <is>
           <t>nein</t>
         </is>
       </c>
-      <c r="I3" s="10" t="inlineStr">
+      <c r="I3" s="11" t="inlineStr">
         <is>
           <t>ja</t>
         </is>
       </c>
-      <c r="J3" s="10" t="inlineStr"/>
-      <c r="K3" s="10" t="inlineStr">
+      <c r="J3" s="11" t="inlineStr"/>
+      <c r="K3" s="11" t="inlineStr">
         <is>
           <t>ganztags</t>
         </is>
       </c>
-      <c r="L3" s="10" t="inlineStr">
+      <c r="L3" s="11" t="inlineStr">
         <is>
           <t>nie</t>
         </is>
       </c>
-      <c r="M3" s="10" t="inlineStr">
+      <c r="M3" s="11" t="inlineStr">
         <is>
           <t>ganztags</t>
         </is>
       </c>
-      <c r="N3" s="10" t="inlineStr">
+      <c r="N3" s="11" t="inlineStr">
         <is>
           <t>ganztags</t>
         </is>
       </c>
-      <c r="O3" s="10" t="inlineStr">
+      <c r="O3" s="11" t="inlineStr">
         <is>
           <t>ganztags</t>
         </is>
       </c>
-      <c r="P3" s="10" t="inlineStr">
+      <c r="P3" s="11" t="inlineStr">
         <is>
           <t>nie</t>
         </is>
       </c>
-      <c r="Q3" s="10" t="inlineStr">
+      <c r="Q3" s="11" t="inlineStr">
         <is>
           <t>nie</t>
         </is>
       </c>
-      <c r="R3" s="10" t="inlineStr">
+      <c r="R3" s="11" t="inlineStr">
         <is>
           <t>Di Berufsschule</t>
         </is>
       </c>
-      <c r="S3" s="10" t="inlineStr">
+      <c r="S3" s="11" t="inlineStr">
         <is>
           <t>Früh</t>
         </is>
       </c>
-      <c r="T3" s="10" t="inlineStr">
+      <c r="T3" s="11" t="inlineStr">
         <is>
           <t>nein</t>
         </is>
       </c>
-      <c r="U3" s="10" t="inlineStr">
+      <c r="U3" s="11" t="inlineStr">
         <is>
           <t>01.11.2026</t>
         </is>
       </c>
-      <c r="V3" s="10" t="inlineStr"/>
-      <c r="W3" s="10" t="inlineStr">
+      <c r="V3" s="11" t="inlineStr"/>
+      <c r="W3" s="11" t="inlineStr">
         <is>
           <t>nicht allein – immer mit Studioleitung</t>
         </is>
@@ -6020,54 +6213,54 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="10" t="inlineStr">
+      <c r="A2" s="11" t="inlineStr">
         <is>
           <t>Lisa M.</t>
         </is>
       </c>
-      <c r="B2" s="10" t="inlineStr">
+      <c r="B2" s="11" t="inlineStr">
         <is>
           <t>Nippes</t>
         </is>
       </c>
-      <c r="C2" s="10" t="inlineStr">
+      <c r="C2" s="11" t="inlineStr">
         <is>
           <t>Spät</t>
         </is>
       </c>
-      <c r="D2" s="10" t="inlineStr">
+      <c r="D2" s="11" t="inlineStr">
         <is>
           <t>Mo, Mi</t>
         </is>
       </c>
-      <c r="E2" s="10" t="inlineStr">
+      <c r="E2" s="11" t="inlineStr">
         <is>
           <t>Beispiel – bitte anpassen</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="10" t="inlineStr">
+      <c r="A3" s="11" t="inlineStr">
         <is>
           <t>Tom K.</t>
         </is>
       </c>
-      <c r="B3" s="10" t="inlineStr">
+      <c r="B3" s="11" t="inlineStr">
         <is>
           <t>Porz</t>
         </is>
       </c>
-      <c r="C3" s="10" t="inlineStr">
+      <c r="C3" s="11" t="inlineStr">
         <is>
           <t>Früh</t>
         </is>
       </c>
-      <c r="D3" s="10" t="inlineStr">
+      <c r="D3" s="11" t="inlineStr">
         <is>
           <t>14.11.2026</t>
         </is>
       </c>
-      <c r="E3" s="10" t="inlineStr">
+      <c r="E3" s="11" t="inlineStr">
         <is>
           <t>Beispiel – Einweisung neues Gerät</t>
         </is>
@@ -6537,58 +6730,58 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="10" t="inlineStr">
+      <c r="A2" s="11" t="inlineStr">
         <is>
           <t>24.12.2026</t>
         </is>
       </c>
-      <c r="B2" s="10" t="inlineStr">
+      <c r="B2" s="11" t="inlineStr">
         <is>
           <t>alle</t>
         </is>
       </c>
-      <c r="C2" s="10" t="inlineStr">
+      <c r="C2" s="11" t="inlineStr">
         <is>
           <t>geschlossen</t>
         </is>
       </c>
-      <c r="D2" s="10" t="inlineStr">
+      <c r="D2" s="11" t="inlineStr">
         <is>
           <t>Spät</t>
         </is>
       </c>
-      <c r="E2" s="10" t="inlineStr"/>
-      <c r="F2" s="10" t="inlineStr">
+      <c r="E2" s="11" t="inlineStr"/>
+      <c r="F2" s="11" t="inlineStr">
         <is>
           <t>Beispiel – Heiligabend nur bis 14 Uhr</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="10" t="inlineStr">
+      <c r="A3" s="11" t="inlineStr">
         <is>
           <t>07.11.2026</t>
         </is>
       </c>
-      <c r="B3" s="10" t="inlineStr">
+      <c r="B3" s="11" t="inlineStr">
         <is>
           <t>Rath</t>
         </is>
       </c>
-      <c r="C3" s="10" t="inlineStr">
+      <c r="C3" s="11" t="inlineStr">
         <is>
           <t>mehr Personen</t>
         </is>
       </c>
-      <c r="D3" s="10" t="inlineStr">
+      <c r="D3" s="11" t="inlineStr">
         <is>
           <t>Samstag</t>
         </is>
       </c>
-      <c r="E3" s="10" t="n">
+      <c r="E3" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="F3" s="10" t="inlineStr">
+      <c r="F3" s="11" t="inlineStr">
         <is>
           <t>Beispiel – Tag der offenen Tür</t>
         </is>
@@ -7261,7 +7454,7 @@
           <t>Wunschfrist (Tag im Vormonat)</t>
         </is>
       </c>
-      <c r="B2" s="7" t="n">
+      <c r="B2" s="8" t="n">
         <v>15</v>
       </c>
       <c r="C2" s="6" t="inlineStr">
@@ -7276,7 +7469,7 @@
           <t>Feiertage geschlossen?</t>
         </is>
       </c>
-      <c r="B3" s="7" t="inlineStr">
+      <c r="B3" s="8" t="inlineStr">
         <is>
           <t>nein</t>
         </is>
@@ -7293,7 +7486,7 @@
           <t>Höchstens Tage am Stück</t>
         </is>
       </c>
-      <c r="B4" s="7" t="n">
+      <c r="B4" s="8" t="n">
         <v>6</v>
       </c>
       <c r="C4" s="6" t="inlineStr">
@@ -7308,7 +7501,7 @@
           <t>Höchstens Wunsch-frei-Tage pro Person und Monat</t>
         </is>
       </c>
-      <c r="B5" s="7" t="n">
+      <c r="B5" s="8" t="n">
         <v>4</v>
       </c>
       <c r="C5" s="6" t="inlineStr">

</xml_diff>

<commit_message>
Schichtplaner: alle Fragen als PDF und in der Vorlage, was von LogX gebraucht wird (Runde 206) (#263)
Claude-Session: https://claude.ai/code/session_01DT8NfaHWD2WwmwkipPurng

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/vorlagen/Schichtplaner-Vorlage.xlsx
+++ b/vorlagen/Schichtplaner-Vorlage.xlsx
@@ -61,13 +61,13 @@
     </font>
     <font>
       <name val="Calibri"/>
-      <b val="1"/>
+      <i val="1"/>
+      <color rgb="0064748B"/>
       <sz val="11"/>
     </font>
     <font>
       <name val="Calibri"/>
-      <i val="1"/>
-      <color rgb="0064748B"/>
+      <b val="1"/>
       <sz val="11"/>
     </font>
   </fonts>
@@ -120,7 +120,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -136,14 +136,17 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -670,13 +673,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D21"/>
+  <dimension ref="A1:E25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
-    <col width="24" customWidth="1" min="2" max="2"/>
-    <col width="70" customWidth="1" min="3" max="3"/>
-    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="62" customWidth="1" min="3" max="3"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
+    <col width="50" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1">
@@ -697,6 +701,11 @@
       </c>
       <c r="D1" s="4" t="inlineStr">
         <is>
+          <t>Heute in der App</t>
+        </is>
+      </c>
+      <c r="E1" s="4" t="inlineStr">
+        <is>
           <t>Antwort</t>
         </is>
       </c>
@@ -707,15 +716,20 @@
       </c>
       <c r="B2" s="6" t="inlineStr">
         <is>
-          <t>Studios und Öffnungszeiten</t>
+          <t>A · Ohne diese Angaben gibt es keinen Plan</t>
         </is>
       </c>
       <c r="C2" s="6" t="inlineStr">
         <is>
-          <t>Welche Öffnungszeiten hat jedes der 14 Studios an welchem Wochentag? (Die Namen stehen schon im Excel – bitte prüfen.) Bitte im Excel im Blatt „Studios“ eintragen.</t>
-        </is>
-      </c>
-      <c r="D2" s="7" t="n"/>
+          <t>Welche Studios sollen im ersten Monat mitgeplant werden – alle 14 oder zum Testen erst eins oder zwei?</t>
+        </is>
+      </c>
+      <c r="D2" s="7" t="inlineStr">
+        <is>
+          <t>Empfehlung: erst ein Studio.</t>
+        </is>
+      </c>
+      <c r="E2" s="8" t="n"/>
     </row>
     <row r="3" ht="48" customHeight="1">
       <c r="A3" s="5" t="n">
@@ -723,15 +737,20 @@
       </c>
       <c r="B3" s="6" t="inlineStr">
         <is>
-          <t>Studios und Öffnungszeiten</t>
+          <t>A · Ohne diese Angaben gibt es keinen Plan</t>
         </is>
       </c>
       <c r="C3" s="6" t="inlineStr">
         <is>
-          <t>An welchen Feiertagen sind die Studios zu? Gibt es Betriebsferien?</t>
-        </is>
-      </c>
-      <c r="D3" s="7" t="n"/>
+          <t>Öffnungszeiten je Studio und Wochentag.</t>
+        </is>
+      </c>
+      <c r="D3" s="7" t="inlineStr">
+        <is>
+          <t>Ins Excel, Blatt „Studios“.</t>
+        </is>
+      </c>
+      <c r="E3" s="8" t="n"/>
     </row>
     <row r="4" ht="48" customHeight="1">
       <c r="A4" s="5" t="n">
@@ -739,15 +758,20 @@
       </c>
       <c r="B4" s="6" t="inlineStr">
         <is>
-          <t>Schichten und Besetzung</t>
+          <t>A · Ohne diese Angaben gibt es keinen Plan</t>
         </is>
       </c>
       <c r="C4" s="6" t="inlineStr">
         <is>
-          <t>Gibt es feste Schichten (z. B. Früh 7–14 Uhr, Spät 14–21 Uhr) oder wechselnde Zeiten? Sind sie in allen Studios gleich? Bitte im Excel im Blatt „Schichten“ eintragen.</t>
-        </is>
-      </c>
-      <c r="D4" s="7" t="n"/>
+          <t>Schichten je Studio: Name, Beginn, Ende, an welchen Wochentagen. Sind sie in allen Studios gleich?</t>
+        </is>
+      </c>
+      <c r="D4" s="7" t="inlineStr">
+        <is>
+          <t>Ins Excel, Blatt „Schichten“. Heute in der Demo: Früh 7–14, Spät 14–21, Samstag 9–14.</t>
+        </is>
+      </c>
+      <c r="E4" s="8" t="n"/>
     </row>
     <row r="5" ht="48" customHeight="1">
       <c r="A5" s="5" t="n">
@@ -755,15 +779,20 @@
       </c>
       <c r="B5" s="6" t="inlineStr">
         <is>
-          <t>Schichten und Besetzung</t>
+          <t>A · Ohne diese Angaben gibt es keinen Plan</t>
         </is>
       </c>
       <c r="C5" s="6" t="inlineStr">
         <is>
-          <t>Wie viele Leute müssen mindestens gleichzeitig im Studio sein? Gibt es Zeiten, Tage oder Studios, an denen es mehr sein müssen (Stoßzeiten)?</t>
-        </is>
-      </c>
-      <c r="D5" s="7" t="n"/>
+          <t>Das Team: eine Zeile pro Person – Name genau wie in der App, Hauptstudio, in welchen Studios sie aushilft, Stunden pro Woche (Minijob: Monatsgrenze).</t>
+        </is>
+      </c>
+      <c r="D5" s="7" t="inlineStr">
+        <is>
+          <t>Ins Excel, Blatt „Mitarbeiter“.</t>
+        </is>
+      </c>
+      <c r="E5" s="8" t="n"/>
     </row>
     <row r="6" ht="48" customHeight="1">
       <c r="A6" s="5" t="n">
@@ -771,15 +800,20 @@
       </c>
       <c r="B6" s="6" t="inlineStr">
         <is>
-          <t>Schichten und Besetzung</t>
+          <t>A · Ohne diese Angaben gibt es keinen Plan</t>
         </is>
       </c>
       <c r="C6" s="6" t="inlineStr">
         <is>
-          <t>Wer darf nicht allein im Studio sein – nur Azubis und Neue, oder auch bestimmte Personen? Und wer zählt als „Begleitung“, damit diese Person nicht mehr allein ist?</t>
-        </is>
-      </c>
-      <c r="D6" s="7" t="n"/>
+          <t>Wer kann wann grundsätzlich nicht? (z. B. „nie Dienstag“, „nur früh“, „Di Uni“)</t>
+        </is>
+      </c>
+      <c r="D6" s="7" t="inlineStr">
+        <is>
+          <t>Ins Excel, Blatt „Mitarbeiter“, Spalten Mo–So und „Sperrzeiten“.</t>
+        </is>
+      </c>
+      <c r="E6" s="8" t="n"/>
     </row>
     <row r="7" ht="48" customHeight="1">
       <c r="A7" s="5" t="n">
@@ -787,15 +821,20 @@
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>Schichten und Besetzung</t>
+          <t>B · Besetzung</t>
         </is>
       </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>Gibt es Aufgaben, die nur bestimmte Personen können (z. B. Probetraining, Kasse, Abschluss am Abend, Erste Hilfe)? Muss in jeder Schicht mindestens eine solche Person da sein?</t>
-        </is>
-      </c>
-      <c r="D7" s="7" t="n"/>
+          <t>Wie viele Personen müssen mindestens gleichzeitig im Studio sein?</t>
+        </is>
+      </c>
+      <c r="D7" s="7" t="inlineStr">
+        <is>
+          <t>Heute: 1 je Schicht.</t>
+        </is>
+      </c>
+      <c r="E7" s="8" t="n"/>
     </row>
     <row r="8" ht="48" customHeight="1">
       <c r="A8" s="5" t="n">
@@ -803,15 +842,20 @@
       </c>
       <c r="B8" s="6" t="inlineStr">
         <is>
-          <t>Schichten und Besetzung</t>
+          <t>B · Besetzung</t>
         </is>
       </c>
       <c r="C8" s="6" t="inlineStr">
         <is>
-          <t>Werden Regionalleiter mit in den Plan eingeteilt, oder stehen sie nur bei Bedarf zur Verfügung?</t>
-        </is>
-      </c>
-      <c r="D8" s="7" t="n"/>
+          <t>Gibt es Stoßzeiten, Tage oder Studios, an denen mehr Leute da sein müssen? Wann, wo, wie viele?</t>
+        </is>
+      </c>
+      <c r="D8" s="7" t="inlineStr">
+        <is>
+          <t>Heute: nur über „Sondertage“ für einzelne Daten.</t>
+        </is>
+      </c>
+      <c r="E8" s="8" t="n"/>
     </row>
     <row r="9" ht="48" customHeight="1">
       <c r="A9" s="5" t="n">
@@ -819,15 +863,20 @@
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>Arbeitszeit und Fairness</t>
+          <t>B · Besetzung</t>
         </is>
       </c>
       <c r="C9" s="6" t="inlineStr">
         <is>
-          <t>Wie lang darf eine Schicht höchstens sein, und ab wann gibt es Pause?</t>
-        </is>
-      </c>
-      <c r="D9" s="7" t="n"/>
+          <t>Wer darf nicht allein im Studio sein (Azubis, Neue, bestimmte Personen)? Und wer zählt als Begleitung?</t>
+        </is>
+      </c>
+      <c r="D9" s="7" t="inlineStr">
+        <is>
+          <t>Heute: Begleitung ist jede Person mit „darf allein: ja“.</t>
+        </is>
+      </c>
+      <c r="E9" s="8" t="n"/>
     </row>
     <row r="10" ht="48" customHeight="1">
       <c r="A10" s="5" t="n">
@@ -835,15 +884,20 @@
       </c>
       <c r="B10" s="6" t="inlineStr">
         <is>
-          <t>Arbeitszeit und Fairness</t>
+          <t>B · Besetzung</t>
         </is>
       </c>
       <c r="C10" s="6" t="inlineStr">
         <is>
-          <t>Wie viele Tage am Stück darf jemand höchstens arbeiten? Gibt es feste freie Tage?</t>
-        </is>
-      </c>
-      <c r="D10" s="7" t="n"/>
+          <t>Muss in bestimmten Schichten jemand mit einer bestimmten Fähigkeit da sein (Probetraining, Kasse, Abschluss am Abend, Erste Hilfe)? In welchen?</t>
+        </is>
+      </c>
+      <c r="D10" s="7" t="inlineStr">
+        <is>
+          <t>Heute: je Schicht eine Fähigkeit („Braucht jemanden mit …“).</t>
+        </is>
+      </c>
+      <c r="E10" s="8" t="n"/>
     </row>
     <row r="11" ht="48" customHeight="1">
       <c r="A11" s="5" t="n">
@@ -851,15 +905,20 @@
       </c>
       <c r="B11" s="6" t="inlineStr">
         <is>
-          <t>Arbeitszeit und Fairness</t>
+          <t>B · Besetzung</t>
         </is>
       </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
-          <t>Wie werden Wochenenden und Feiertage verteilt – reihum, oder hat jemand fest frei?</t>
-        </is>
-      </c>
-      <c r="D11" s="7" t="n"/>
+          <t>Werden Studioleitungen und Regionalleiter fest eingeplant oder nur bei Bedarf?</t>
+        </is>
+      </c>
+      <c r="D11" s="7" t="inlineStr">
+        <is>
+          <t>Heute: wie alle anderen, wenn sie im Blatt „Mitarbeiter“ stehen.</t>
+        </is>
+      </c>
+      <c r="E11" s="8" t="n"/>
     </row>
     <row r="12" ht="48" customHeight="1">
       <c r="A12" s="5" t="n">
@@ -867,15 +926,20 @@
       </c>
       <c r="B12" s="6" t="inlineStr">
         <is>
-          <t>Arbeitszeit und Fairness</t>
+          <t>C · Arbeitszeit</t>
         </is>
       </c>
       <c r="C12" s="6" t="inlineStr">
         <is>
-          <t>Gibt es Mitarbeiter unter 18 Jahren? Für sie gelten strengere Regeln (z. B. keine späten Schichten).</t>
-        </is>
-      </c>
-      <c r="D12" s="7" t="n"/>
+          <t>Wie lang darf eine Schicht höchstens sein, und ab wann gibt es Pause?</t>
+        </is>
+      </c>
+      <c r="D12" s="7" t="inlineStr">
+        <is>
+          <t>Heute: wird nicht geprüft.</t>
+        </is>
+      </c>
+      <c r="E12" s="8" t="n"/>
     </row>
     <row r="13" ht="48" customHeight="1">
       <c r="A13" s="5" t="n">
@@ -883,15 +947,20 @@
       </c>
       <c r="B13" s="6" t="inlineStr">
         <is>
-          <t>Arbeitszeit und Fairness</t>
+          <t>C · Arbeitszeit</t>
         </is>
       </c>
       <c r="C13" s="6" t="inlineStr">
         <is>
-          <t>Minijobs: Gilt pro Person eine feste Höchstzahl an Stunden im Monat? Wenn nein: Wie hoch ist der Stundenlohn, damit die Maschine die Grenze ausrechnen kann?</t>
-        </is>
-      </c>
-      <c r="D13" s="7" t="n"/>
+          <t>Wie viele Tage am Stück darf jemand höchstens arbeiten?</t>
+        </is>
+      </c>
+      <c r="D13" s="7" t="inlineStr">
+        <is>
+          <t>Heute: 6.</t>
+        </is>
+      </c>
+      <c r="E13" s="8" t="n"/>
     </row>
     <row r="14" ht="48" customHeight="1">
       <c r="A14" s="5" t="n">
@@ -899,15 +968,20 @@
       </c>
       <c r="B14" s="6" t="inlineStr">
         <is>
-          <t>Wünsche und Konflikte</t>
+          <t>C · Arbeitszeit</t>
         </is>
       </c>
       <c r="C14" s="6" t="inlineStr">
         <is>
-          <t>Was hat Vorrang, wenn sich etwas beisst? Bitte in eine Reihenfolge bringen: Besetzung · vereinbarte Stunden · Wünsche der Mitarbeiter · Fairness.</t>
-        </is>
-      </c>
-      <c r="D14" s="7" t="n"/>
+          <t>Höchstens wie viele Tage pro Woche – für alle gleich oder je Person?</t>
+        </is>
+      </c>
+      <c r="D14" s="7" t="inlineStr">
+        <is>
+          <t>Heute: je Person im Excel, sonst ohne Grenze.</t>
+        </is>
+      </c>
+      <c r="E14" s="8" t="n"/>
     </row>
     <row r="15" ht="48" customHeight="1">
       <c r="A15" s="5" t="n">
@@ -915,15 +989,20 @@
       </c>
       <c r="B15" s="6" t="inlineStr">
         <is>
-          <t>Wünsche und Konflikte</t>
+          <t>C · Arbeitszeit</t>
         </is>
       </c>
       <c r="C15" s="6" t="inlineStr">
         <is>
-          <t>Bis wann vor dem Monat müssen die Wünsche eingetragen sein (z. B. bis zum 15. des Vormonats)?</t>
-        </is>
-      </c>
-      <c r="D15" s="7" t="n"/>
+          <t>Gibt es Mitarbeiter unter 18?</t>
+        </is>
+      </c>
+      <c r="D15" s="7" t="inlineStr">
+        <is>
+          <t>Wenn ja, gilt automatisch: nur 6–20 Uhr, höchstens 8 Stunden.</t>
+        </is>
+      </c>
+      <c r="E15" s="8" t="n"/>
     </row>
     <row r="16" ht="48" customHeight="1">
       <c r="A16" s="5" t="n">
@@ -931,15 +1010,20 @@
       </c>
       <c r="B16" s="6" t="inlineStr">
         <is>
-          <t>Wünsche und Konflikte</t>
+          <t>C · Arbeitszeit</t>
         </is>
       </c>
       <c r="C16" s="6" t="inlineStr">
         <is>
-          <t>Wie viele Wunsch-frei-Tage darf jeder pro Monat angeben?</t>
-        </is>
-      </c>
-      <c r="D16" s="7" t="n"/>
+          <t>Feiertage in NRW: geschlossen oder offen? Gibt es Betriebsferien?</t>
+        </is>
+      </c>
+      <c r="D16" s="7" t="inlineStr">
+        <is>
+          <t>Heute: offen (umschaltbar).</t>
+        </is>
+      </c>
+      <c r="E16" s="8" t="n"/>
     </row>
     <row r="17" ht="48" customHeight="1">
       <c r="A17" s="5" t="n">
@@ -947,15 +1031,20 @@
       </c>
       <c r="B17" s="6" t="inlineStr">
         <is>
-          <t>Wünsche und Konflikte</t>
+          <t>D · Wünsche und Fairness</t>
         </is>
       </c>
       <c r="C17" s="6" t="inlineStr">
         <is>
-          <t>Wenn eine Schicht nicht zu besetzen ist: Soll die Maschine nur die Lücke melden oder gleich vorschlagen, wen man fragen könnte?</t>
-        </is>
-      </c>
-      <c r="D17" s="7" t="n"/>
+          <t>Bis zum wievielten des Vormonats müssen Wünsche eingetragen sein?</t>
+        </is>
+      </c>
+      <c r="D17" s="7" t="inlineStr">
+        <is>
+          <t>Heute: bis zum 15.</t>
+        </is>
+      </c>
+      <c r="E17" s="8" t="n"/>
     </row>
     <row r="18" ht="48" customHeight="1">
       <c r="A18" s="5" t="n">
@@ -963,15 +1052,20 @@
       </c>
       <c r="B18" s="6" t="inlineStr">
         <is>
-          <t>Ablauf und LogX</t>
+          <t>D · Wünsche und Fairness</t>
         </is>
       </c>
       <c r="C18" s="6" t="inlineStr">
         <is>
-          <t>Wer prüft und veröffentlicht den Plan – nur Sie, oder auch die Studioleiter für ihre Studios?</t>
-        </is>
-      </c>
-      <c r="D18" s="7" t="n"/>
+          <t>Wie viele Wunsch-frei-Tage darf jede Person im Monat angeben?</t>
+        </is>
+      </c>
+      <c r="D18" s="7" t="inlineStr">
+        <is>
+          <t>Heute: keine Grenze.</t>
+        </is>
+      </c>
+      <c r="E18" s="8" t="n"/>
     </row>
     <row r="19" ht="48" customHeight="1">
       <c r="A19" s="5" t="n">
@@ -979,15 +1073,20 @@
       </c>
       <c r="B19" s="6" t="inlineStr">
         <is>
-          <t>Ablauf und LogX</t>
+          <t>D · Wünsche und Fairness</t>
         </is>
       </c>
       <c r="C19" s="6" t="inlineStr">
         <is>
-          <t>Wie weit im Voraus soll der Plan fertig sein (z. B. am 20. für den nächsten Monat)?</t>
-        </is>
-      </c>
-      <c r="D19" s="7" t="n"/>
+          <t>Was hat Vorrang, wenn es sich beisst? Bitte in eine Reihenfolge: Besetzung · vereinbarte Stunden · Wünsche · Fairness.</t>
+        </is>
+      </c>
+      <c r="D19" s="7" t="inlineStr">
+        <is>
+          <t>Heute: Besetzung zuerst; ein Wunsch wird nur als Rückfrage gebrochen.</t>
+        </is>
+      </c>
+      <c r="E19" s="8" t="n"/>
     </row>
     <row r="20" ht="48" customHeight="1">
       <c r="A20" s="5" t="n">
@@ -995,15 +1094,20 @@
       </c>
       <c r="B20" s="6" t="inlineStr">
         <is>
-          <t>Ablauf und LogX</t>
+          <t>D · Wünsche und Fairness</t>
         </is>
       </c>
       <c r="C20" s="6" t="inlineStr">
         <is>
-          <t>Wie wird heute in LogX eingetragen? Hilfreich wären Bildschirmfotos und ein exportierter alter Plan.</t>
-        </is>
-      </c>
-      <c r="D20" s="7" t="n"/>
+          <t>Wochenenden: reihum verteilen, oder hat jemand fest frei?</t>
+        </is>
+      </c>
+      <c r="D20" s="7" t="inlineStr">
+        <is>
+          <t>Heute: reihum, so gleich wie möglich.</t>
+        </is>
+      </c>
+      <c r="E20" s="8" t="n"/>
     </row>
     <row r="21" ht="48" customHeight="1">
       <c r="A21" s="5" t="n">
@@ -1011,15 +1115,104 @@
       </c>
       <c r="B21" s="6" t="inlineStr">
         <is>
-          <t>Ablauf und LogX</t>
+          <t>D · Wünsche und Fairness</t>
         </is>
       </c>
       <c r="C21" s="6" t="inlineStr">
         <is>
-          <t>Kann LogX Dateien importieren oder exportieren (Excel/CSV)? Gibt es eine Mitarbeiterliste zum Exportieren?</t>
-        </is>
-      </c>
-      <c r="D21" s="7" t="n"/>
+          <t>Fällt jemand aus: nur die Lücke melden oder gleich vorschlagen, wen man fragen kann?</t>
+        </is>
+      </c>
+      <c r="D21" s="7" t="inlineStr">
+        <is>
+          <t>Heute: bis zu drei Vorschläge.</t>
+        </is>
+      </c>
+      <c r="E21" s="8" t="n"/>
+    </row>
+    <row r="22" ht="48" customHeight="1">
+      <c r="A22" s="5" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" s="6" t="inlineStr">
+        <is>
+          <t>E · Ablauf</t>
+        </is>
+      </c>
+      <c r="C22" s="6" t="inlineStr">
+        <is>
+          <t>Wer erstellt und veröffentlicht den Plan – nur die Geschäftsführung oder auch die Studioleitung für ihr Studio?</t>
+        </is>
+      </c>
+      <c r="D22" s="7" t="inlineStr">
+        <is>
+          <t>Heute: nur die Geschäftsführung.</t>
+        </is>
+      </c>
+      <c r="E22" s="8" t="n"/>
+    </row>
+    <row r="23" ht="48" customHeight="1">
+      <c r="A23" s="5" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" s="6" t="inlineStr">
+        <is>
+          <t>E · Ablauf</t>
+        </is>
+      </c>
+      <c r="C23" s="6" t="inlineStr">
+        <is>
+          <t>Bis wann muss der Plan für den nächsten Monat fertig sein (z. B. am 20.)?</t>
+        </is>
+      </c>
+      <c r="D23" s="7" t="inlineStr">
+        <is>
+          <t>Heute: keine Frist.</t>
+        </is>
+      </c>
+      <c r="E23" s="8" t="n"/>
+    </row>
+    <row r="24" ht="48" customHeight="1">
+      <c r="A24" s="5" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" s="6" t="inlineStr">
+        <is>
+          <t>E · Ablauf</t>
+        </is>
+      </c>
+      <c r="C24" s="6" t="inlineStr">
+        <is>
+          <t>Muss die Leitung jeden Schichttausch bestätigen?</t>
+        </is>
+      </c>
+      <c r="D24" s="7" t="inlineStr">
+        <is>
+          <t>Heute: ja.</t>
+        </is>
+      </c>
+      <c r="E24" s="8" t="n"/>
+    </row>
+    <row r="25" ht="48" customHeight="1">
+      <c r="A25" s="5" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" s="6" t="inlineStr">
+        <is>
+          <t>E · Ablauf</t>
+        </is>
+      </c>
+      <c r="C25" s="6" t="inlineStr">
+        <is>
+          <t>Wird der Plan danach noch in LogX eingetragen? (Was ich dafür brauche: letzte Seite)</t>
+        </is>
+      </c>
+      <c r="D25" s="7" t="inlineStr">
+        <is>
+          <t>Heute: „Für LogX kopieren“ legt eine Tabelle in die Zwischenablage.</t>
+        </is>
+      </c>
+      <c r="E25" s="8" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1115,7 +1308,7 @@
       </c>
     </row>
     <row r="2" ht="22" customHeight="1">
-      <c r="A2" s="8" t="inlineStr">
+      <c r="A2" s="9" t="inlineStr">
         <is>
           <t>Longerich</t>
         </is>
@@ -1132,7 +1325,7 @@
       <c r="K2" s="6" t="n"/>
     </row>
     <row r="3" ht="22" customHeight="1">
-      <c r="A3" s="8" t="inlineStr">
+      <c r="A3" s="9" t="inlineStr">
         <is>
           <t>Nippes</t>
         </is>
@@ -1149,7 +1342,7 @@
       <c r="K3" s="6" t="n"/>
     </row>
     <row r="4" ht="22" customHeight="1">
-      <c r="A4" s="8" t="inlineStr">
+      <c r="A4" s="9" t="inlineStr">
         <is>
           <t>Ebertplatz</t>
         </is>
@@ -1166,7 +1359,7 @@
       <c r="K4" s="6" t="n"/>
     </row>
     <row r="5" ht="22" customHeight="1">
-      <c r="A5" s="8" t="inlineStr">
+      <c r="A5" s="9" t="inlineStr">
         <is>
           <t>Rath</t>
         </is>
@@ -1183,7 +1376,7 @@
       <c r="K5" s="6" t="n"/>
     </row>
     <row r="6" ht="22" customHeight="1">
-      <c r="A6" s="8" t="inlineStr">
+      <c r="A6" s="9" t="inlineStr">
         <is>
           <t>Porz</t>
         </is>
@@ -1200,7 +1393,7 @@
       <c r="K6" s="6" t="n"/>
     </row>
     <row r="7" ht="22" customHeight="1">
-      <c r="A7" s="8" t="inlineStr">
+      <c r="A7" s="9" t="inlineStr">
         <is>
           <t>Rondorf</t>
         </is>
@@ -1217,7 +1410,7 @@
       <c r="K7" s="6" t="n"/>
     </row>
     <row r="8" ht="22" customHeight="1">
-      <c r="A8" s="8" t="inlineStr">
+      <c r="A8" s="9" t="inlineStr">
         <is>
           <t>Hürth</t>
         </is>
@@ -1234,7 +1427,7 @@
       <c r="K8" s="6" t="n"/>
     </row>
     <row r="9" ht="22" customHeight="1">
-      <c r="A9" s="8" t="inlineStr">
+      <c r="A9" s="9" t="inlineStr">
         <is>
           <t>Brühl</t>
         </is>
@@ -1251,7 +1444,7 @@
       <c r="K9" s="6" t="n"/>
     </row>
     <row r="10" ht="22" customHeight="1">
-      <c r="A10" s="8" t="inlineStr">
+      <c r="A10" s="9" t="inlineStr">
         <is>
           <t>Niederkassel Mondorf</t>
         </is>
@@ -1268,7 +1461,7 @@
       <c r="K10" s="6" t="n"/>
     </row>
     <row r="11" ht="22" customHeight="1">
-      <c r="A11" s="8" t="inlineStr">
+      <c r="A11" s="9" t="inlineStr">
         <is>
           <t>Refrath</t>
         </is>
@@ -1285,7 +1478,7 @@
       <c r="K11" s="6" t="n"/>
     </row>
     <row r="12" ht="22" customHeight="1">
-      <c r="A12" s="8" t="inlineStr">
+      <c r="A12" s="9" t="inlineStr">
         <is>
           <t>Overath</t>
         </is>
@@ -1302,7 +1495,7 @@
       <c r="K12" s="6" t="n"/>
     </row>
     <row r="13" ht="22" customHeight="1">
-      <c r="A13" s="8" t="inlineStr">
+      <c r="A13" s="9" t="inlineStr">
         <is>
           <t>Marialinden</t>
         </is>
@@ -1319,7 +1512,7 @@
       <c r="K13" s="6" t="n"/>
     </row>
     <row r="14" ht="22" customHeight="1">
-      <c r="A14" s="8" t="inlineStr">
+      <c r="A14" s="9" t="inlineStr">
         <is>
           <t>Rösrath</t>
         </is>
@@ -1336,7 +1529,7 @@
       <c r="K14" s="6" t="n"/>
     </row>
     <row r="15" ht="22" customHeight="1">
-      <c r="A15" s="8" t="inlineStr">
+      <c r="A15" s="9" t="inlineStr">
         <is>
           <t>Seelscheid</t>
         </is>
@@ -1353,7 +1546,7 @@
       <c r="K15" s="6" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="9" t="inlineStr">
+      <c r="A17" s="10" t="inlineStr">
         <is>
           <t>Beispiel für eine Zeile: Mo 07:00–21:00 · mindestens 1 · „Mo–Do 16–20 Uhr 2 Personen“ · „Sa nur bis 14 Uhr“</t>
         </is>
@@ -1434,112 +1627,112 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="10" t="inlineStr">
+      <c r="A2" s="11" t="inlineStr">
         <is>
           <t>alle</t>
         </is>
       </c>
-      <c r="B2" s="10" t="inlineStr">
+      <c r="B2" s="11" t="inlineStr">
         <is>
           <t>Früh</t>
         </is>
       </c>
-      <c r="C2" s="10" t="inlineStr">
+      <c r="C2" s="11" t="inlineStr">
         <is>
           <t>07:00</t>
         </is>
       </c>
-      <c r="D2" s="10" t="inlineStr">
+      <c r="D2" s="11" t="inlineStr">
         <is>
           <t>14:00</t>
         </is>
       </c>
-      <c r="E2" s="10" t="inlineStr">
+      <c r="E2" s="11" t="inlineStr">
         <is>
           <t>Mo–Fr</t>
         </is>
       </c>
-      <c r="F2" s="10" t="n">
+      <c r="F2" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="G2" s="10" t="inlineStr"/>
-      <c r="H2" s="10" t="inlineStr">
+      <c r="G2" s="11" t="inlineStr"/>
+      <c r="H2" s="11" t="inlineStr">
         <is>
           <t>Beispiel – bitte anpassen</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="10" t="inlineStr">
+      <c r="A3" s="11" t="inlineStr">
         <is>
           <t>alle</t>
         </is>
       </c>
-      <c r="B3" s="10" t="inlineStr">
+      <c r="B3" s="11" t="inlineStr">
         <is>
           <t>Spät</t>
         </is>
       </c>
-      <c r="C3" s="10" t="inlineStr">
+      <c r="C3" s="11" t="inlineStr">
         <is>
           <t>14:00</t>
         </is>
       </c>
-      <c r="D3" s="10" t="inlineStr">
+      <c r="D3" s="11" t="inlineStr">
         <is>
           <t>21:00</t>
         </is>
       </c>
-      <c r="E3" s="10" t="inlineStr">
+      <c r="E3" s="11" t="inlineStr">
         <is>
           <t>Mo–Fr</t>
         </is>
       </c>
-      <c r="F3" s="10" t="n">
+      <c r="F3" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="G3" s="10" t="inlineStr">
+      <c r="G3" s="11" t="inlineStr">
         <is>
           <t>Abschluss</t>
         </is>
       </c>
-      <c r="H3" s="10" t="inlineStr">
+      <c r="H3" s="11" t="inlineStr">
         <is>
           <t>Beispiel – bitte anpassen</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="10" t="inlineStr">
+      <c r="A4" s="11" t="inlineStr">
         <is>
           <t>alle</t>
         </is>
       </c>
-      <c r="B4" s="10" t="inlineStr">
+      <c r="B4" s="11" t="inlineStr">
         <is>
           <t>Samstag</t>
         </is>
       </c>
-      <c r="C4" s="10" t="inlineStr">
+      <c r="C4" s="11" t="inlineStr">
         <is>
           <t>09:00</t>
         </is>
       </c>
-      <c r="D4" s="10" t="inlineStr">
+      <c r="D4" s="11" t="inlineStr">
         <is>
           <t>14:00</t>
         </is>
       </c>
-      <c r="E4" s="10" t="inlineStr">
+      <c r="E4" s="11" t="inlineStr">
         <is>
           <t>Sa</t>
         </is>
       </c>
-      <c r="F4" s="10" t="n">
+      <c r="F4" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="G4" s="10" t="inlineStr"/>
-      <c r="H4" s="10" t="inlineStr">
+      <c r="G4" s="11" t="inlineStr"/>
+      <c r="H4" s="11" t="inlineStr">
         <is>
           <t>Beispiel – bitte anpassen</t>
         </is>
@@ -2079,194 +2272,194 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="10" t="inlineStr">
+      <c r="A2" s="11" t="inlineStr">
         <is>
           <t>Beispiel: Lisa M.</t>
         </is>
       </c>
-      <c r="B2" s="10" t="inlineStr">
+      <c r="B2" s="11" t="inlineStr">
         <is>
           <t>Minijob</t>
         </is>
       </c>
-      <c r="C2" s="10" t="inlineStr">
+      <c r="C2" s="11" t="inlineStr">
         <is>
           <t>Nippes</t>
         </is>
       </c>
-      <c r="D2" s="10" t="inlineStr">
+      <c r="D2" s="11" t="inlineStr">
         <is>
           <t>Longerich, Ebertplatz</t>
         </is>
       </c>
-      <c r="E2" s="10" t="inlineStr"/>
-      <c r="F2" s="10" t="n">
+      <c r="E2" s="11" t="inlineStr"/>
+      <c r="F2" s="11" t="n">
         <v>40</v>
       </c>
-      <c r="G2" s="10" t="n">
+      <c r="G2" s="11" t="n">
         <v>3</v>
       </c>
-      <c r="H2" s="10" t="inlineStr">
+      <c r="H2" s="11" t="inlineStr">
         <is>
           <t>ja</t>
         </is>
       </c>
-      <c r="I2" s="10" t="inlineStr">
+      <c r="I2" s="11" t="inlineStr">
         <is>
           <t>nein</t>
         </is>
       </c>
-      <c r="J2" s="10" t="inlineStr">
+      <c r="J2" s="11" t="inlineStr">
         <is>
           <t>Probetraining</t>
         </is>
       </c>
-      <c r="K2" s="10" t="inlineStr">
+      <c r="K2" s="11" t="inlineStr">
         <is>
           <t>nur spät</t>
         </is>
       </c>
-      <c r="L2" s="10" t="inlineStr">
+      <c r="L2" s="11" t="inlineStr">
         <is>
           <t>nie</t>
         </is>
       </c>
-      <c r="M2" s="10" t="inlineStr">
+      <c r="M2" s="11" t="inlineStr">
         <is>
           <t>nur spät</t>
         </is>
       </c>
-      <c r="N2" s="10" t="inlineStr">
+      <c r="N2" s="11" t="inlineStr">
         <is>
           <t>nie</t>
         </is>
       </c>
-      <c r="O2" s="10" t="inlineStr">
+      <c r="O2" s="11" t="inlineStr">
         <is>
           <t>ganztags</t>
         </is>
       </c>
-      <c r="P2" s="10" t="inlineStr">
+      <c r="P2" s="11" t="inlineStr">
         <is>
           <t>ganztags</t>
         </is>
       </c>
-      <c r="Q2" s="10" t="inlineStr">
+      <c r="Q2" s="11" t="inlineStr">
         <is>
           <t>nie</t>
         </is>
       </c>
-      <c r="R2" s="10" t="inlineStr"/>
-      <c r="S2" s="10" t="inlineStr">
+      <c r="R2" s="11" t="inlineStr"/>
+      <c r="S2" s="11" t="inlineStr">
         <is>
           <t>Spät</t>
         </is>
       </c>
-      <c r="T2" s="10" t="inlineStr">
+      <c r="T2" s="11" t="inlineStr">
         <is>
           <t>ja</t>
         </is>
       </c>
-      <c r="U2" s="10" t="inlineStr"/>
-      <c r="V2" s="10" t="inlineStr"/>
-      <c r="W2" s="10" t="inlineStr">
+      <c r="U2" s="11" t="inlineStr"/>
+      <c r="V2" s="11" t="inlineStr"/>
+      <c r="W2" s="11" t="inlineStr">
         <is>
           <t>samstags nur alle zwei Wochen</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="10" t="inlineStr">
+      <c r="A3" s="11" t="inlineStr">
         <is>
           <t>Beispiel: Tom K.</t>
         </is>
       </c>
-      <c r="B3" s="10" t="inlineStr">
+      <c r="B3" s="11" t="inlineStr">
         <is>
           <t>Azubi</t>
         </is>
       </c>
-      <c r="C3" s="10" t="inlineStr">
+      <c r="C3" s="11" t="inlineStr">
         <is>
           <t>Porz</t>
         </is>
       </c>
-      <c r="D3" s="10" t="inlineStr"/>
-      <c r="E3" s="10" t="n">
+      <c r="D3" s="11" t="inlineStr"/>
+      <c r="E3" s="11" t="n">
         <v>40</v>
       </c>
-      <c r="F3" s="10" t="inlineStr"/>
-      <c r="G3" s="10" t="n">
+      <c r="F3" s="11" t="inlineStr"/>
+      <c r="G3" s="11" t="n">
         <v>5</v>
       </c>
-      <c r="H3" s="10" t="inlineStr">
+      <c r="H3" s="11" t="inlineStr">
         <is>
           <t>nein</t>
         </is>
       </c>
-      <c r="I3" s="10" t="inlineStr">
+      <c r="I3" s="11" t="inlineStr">
         <is>
           <t>ja</t>
         </is>
       </c>
-      <c r="J3" s="10" t="inlineStr"/>
-      <c r="K3" s="10" t="inlineStr">
+      <c r="J3" s="11" t="inlineStr"/>
+      <c r="K3" s="11" t="inlineStr">
         <is>
           <t>ganztags</t>
         </is>
       </c>
-      <c r="L3" s="10" t="inlineStr">
+      <c r="L3" s="11" t="inlineStr">
         <is>
           <t>nie</t>
         </is>
       </c>
-      <c r="M3" s="10" t="inlineStr">
+      <c r="M3" s="11" t="inlineStr">
         <is>
           <t>ganztags</t>
         </is>
       </c>
-      <c r="N3" s="10" t="inlineStr">
+      <c r="N3" s="11" t="inlineStr">
         <is>
           <t>ganztags</t>
         </is>
       </c>
-      <c r="O3" s="10" t="inlineStr">
+      <c r="O3" s="11" t="inlineStr">
         <is>
           <t>ganztags</t>
         </is>
       </c>
-      <c r="P3" s="10" t="inlineStr">
+      <c r="P3" s="11" t="inlineStr">
         <is>
           <t>nie</t>
         </is>
       </c>
-      <c r="Q3" s="10" t="inlineStr">
+      <c r="Q3" s="11" t="inlineStr">
         <is>
           <t>nie</t>
         </is>
       </c>
-      <c r="R3" s="10" t="inlineStr">
+      <c r="R3" s="11" t="inlineStr">
         <is>
           <t>Di Berufsschule</t>
         </is>
       </c>
-      <c r="S3" s="10" t="inlineStr">
+      <c r="S3" s="11" t="inlineStr">
         <is>
           <t>Früh</t>
         </is>
       </c>
-      <c r="T3" s="10" t="inlineStr">
+      <c r="T3" s="11" t="inlineStr">
         <is>
           <t>nein</t>
         </is>
       </c>
-      <c r="U3" s="10" t="inlineStr">
+      <c r="U3" s="11" t="inlineStr">
         <is>
           <t>01.11.2026</t>
         </is>
       </c>
-      <c r="V3" s="10" t="inlineStr"/>
-      <c r="W3" s="10" t="inlineStr">
+      <c r="V3" s="11" t="inlineStr"/>
+      <c r="W3" s="11" t="inlineStr">
         <is>
           <t>nicht allein – immer mit Studioleitung</t>
         </is>
@@ -6020,54 +6213,54 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="10" t="inlineStr">
+      <c r="A2" s="11" t="inlineStr">
         <is>
           <t>Lisa M.</t>
         </is>
       </c>
-      <c r="B2" s="10" t="inlineStr">
+      <c r="B2" s="11" t="inlineStr">
         <is>
           <t>Nippes</t>
         </is>
       </c>
-      <c r="C2" s="10" t="inlineStr">
+      <c r="C2" s="11" t="inlineStr">
         <is>
           <t>Spät</t>
         </is>
       </c>
-      <c r="D2" s="10" t="inlineStr">
+      <c r="D2" s="11" t="inlineStr">
         <is>
           <t>Mo, Mi</t>
         </is>
       </c>
-      <c r="E2" s="10" t="inlineStr">
+      <c r="E2" s="11" t="inlineStr">
         <is>
           <t>Beispiel – bitte anpassen</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="10" t="inlineStr">
+      <c r="A3" s="11" t="inlineStr">
         <is>
           <t>Tom K.</t>
         </is>
       </c>
-      <c r="B3" s="10" t="inlineStr">
+      <c r="B3" s="11" t="inlineStr">
         <is>
           <t>Porz</t>
         </is>
       </c>
-      <c r="C3" s="10" t="inlineStr">
+      <c r="C3" s="11" t="inlineStr">
         <is>
           <t>Früh</t>
         </is>
       </c>
-      <c r="D3" s="10" t="inlineStr">
+      <c r="D3" s="11" t="inlineStr">
         <is>
           <t>14.11.2026</t>
         </is>
       </c>
-      <c r="E3" s="10" t="inlineStr">
+      <c r="E3" s="11" t="inlineStr">
         <is>
           <t>Beispiel – Einweisung neues Gerät</t>
         </is>
@@ -6537,58 +6730,58 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="10" t="inlineStr">
+      <c r="A2" s="11" t="inlineStr">
         <is>
           <t>24.12.2026</t>
         </is>
       </c>
-      <c r="B2" s="10" t="inlineStr">
+      <c r="B2" s="11" t="inlineStr">
         <is>
           <t>alle</t>
         </is>
       </c>
-      <c r="C2" s="10" t="inlineStr">
+      <c r="C2" s="11" t="inlineStr">
         <is>
           <t>geschlossen</t>
         </is>
       </c>
-      <c r="D2" s="10" t="inlineStr">
+      <c r="D2" s="11" t="inlineStr">
         <is>
           <t>Spät</t>
         </is>
       </c>
-      <c r="E2" s="10" t="inlineStr"/>
-      <c r="F2" s="10" t="inlineStr">
+      <c r="E2" s="11" t="inlineStr"/>
+      <c r="F2" s="11" t="inlineStr">
         <is>
           <t>Beispiel – Heiligabend nur bis 14 Uhr</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="10" t="inlineStr">
+      <c r="A3" s="11" t="inlineStr">
         <is>
           <t>07.11.2026</t>
         </is>
       </c>
-      <c r="B3" s="10" t="inlineStr">
+      <c r="B3" s="11" t="inlineStr">
         <is>
           <t>Rath</t>
         </is>
       </c>
-      <c r="C3" s="10" t="inlineStr">
+      <c r="C3" s="11" t="inlineStr">
         <is>
           <t>mehr Personen</t>
         </is>
       </c>
-      <c r="D3" s="10" t="inlineStr">
+      <c r="D3" s="11" t="inlineStr">
         <is>
           <t>Samstag</t>
         </is>
       </c>
-      <c r="E3" s="10" t="n">
+      <c r="E3" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="F3" s="10" t="inlineStr">
+      <c r="F3" s="11" t="inlineStr">
         <is>
           <t>Beispiel – Tag der offenen Tür</t>
         </is>
@@ -7261,7 +7454,7 @@
           <t>Wunschfrist (Tag im Vormonat)</t>
         </is>
       </c>
-      <c r="B2" s="7" t="n">
+      <c r="B2" s="8" t="n">
         <v>15</v>
       </c>
       <c r="C2" s="6" t="inlineStr">
@@ -7276,7 +7469,7 @@
           <t>Feiertage geschlossen?</t>
         </is>
       </c>
-      <c r="B3" s="7" t="inlineStr">
+      <c r="B3" s="8" t="inlineStr">
         <is>
           <t>nein</t>
         </is>
@@ -7293,7 +7486,7 @@
           <t>Höchstens Tage am Stück</t>
         </is>
       </c>
-      <c r="B4" s="7" t="n">
+      <c r="B4" s="8" t="n">
         <v>6</v>
       </c>
       <c r="C4" s="6" t="inlineStr">
@@ -7308,7 +7501,7 @@
           <t>Höchstens Wunsch-frei-Tage pro Person und Monat</t>
         </is>
       </c>
-      <c r="B5" s="7" t="n">
+      <c r="B5" s="8" t="n">
         <v>4</v>
       </c>
       <c r="C5" s="6" t="inlineStr">

</xml_diff>